<commit_message>
NPB自動更新(1軍): 2026-09-13 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-13.xlsx
+++ b/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-13.xlsx
@@ -96227,17 +96227,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>正木 智也</t>
+          <t>髙橋 宏斗</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ソフトバンク</t>
+          <t>中日</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2本塁打4打点猛打賞の大活躍。6回裏に2本目のホームランを放ち勝利に貢献。</t>
+          <t>9回を投げ被安打4、12奪三振の快投で相手打線を完封し、チームを勝利に導いた。</t>
         </is>
       </c>
     </row>
@@ -96252,17 +96252,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>髙橋 宏斗</t>
+          <t>正木 智也</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>中日</t>
+          <t>ソフトバンク</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>9回を投げ被安打4、12奪三振無失点の快投で、相手打線を完全に封じ込めた。</t>
+          <t>4回裏に勝ち越し2ラン、6回裏にもソロを放ち、チームの勝利に大きく貢献した。</t>
         </is>
       </c>
     </row>
@@ -96277,17 +96277,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>才木 浩人</t>
+          <t>細川 成也</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>阪神</t>
+          <t>中日</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>髙橋宏斗との投手戦を演じ、9回9奪三振無失点の好投で試合を支配した。</t>
+          <t>延長11回表にレフトへの先制タイムリーツーベースを放ち、均衡を破る決勝打となった。</t>
         </is>
       </c>
     </row>
@@ -96302,17 +96302,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高橋 奎二</t>
+          <t>才木 浩人</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ヤクルト</t>
+          <t>阪神</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6回を投げ被安打4、8奪三振無失点の力投で、試合の主導権を握った。</t>
+          <t>髙橋宏斗との投手戦を繰り広げ、9回を投げ被安打3、9奪三振の力投で中日打線を無失点に抑えた。</t>
         </is>
       </c>
     </row>
@@ -96327,17 +96327,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>細川 成也</t>
+          <t>佐野 恵太</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>中日</t>
+          <t>DeNA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>延長11回表に均衡を破る先制タイムリーツーベースを放ち、チームを勝利に導いた。</t>
+          <t>1回裏にライトスタンドへ先制の満塁ホームランを放ち、試合の主導権を握る一打となった。</t>
         </is>
       </c>
     </row>
@@ -96352,17 +96352,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>佐野 恵太</t>
+          <t>水野 達稀</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DeNA</t>
+          <t>日本ハム</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1回裏にライトスタンドへ先制満塁ホームランを放ち、試合の序盤で主導権を握った。</t>
+          <t>3安打猛打賞に加え、2盗塁も記録し、攻撃の起点としてチームの大量得点に貢献した。</t>
         </is>
       </c>
     </row>

</xml_diff>